<commit_message>
Update industrial sector (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/industrial sector (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/industrial sector (VDS_s) 0.xlsx
@@ -597,968 +597,968 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2">
         <v>2021</v>
       </c>
       <c r="D2" s="3">
-        <v>496312.33844584553</v>
+        <v>2688475.9724428668</v>
       </c>
       <c r="E2" s="3">
-        <v>6058.6276942799996</v>
+        <v>22918.622383440001</v>
       </c>
       <c r="F2" s="4">
-        <v>1.149126975828702E-3</v>
+        <v>1.411209606183382E-2</v>
       </c>
       <c r="G2" s="4">
-        <v>4.3326889923906344E-3</v>
+        <v>6.7540592802753808E-4</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="5">
-        <v>2023</v>
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2022</v>
       </c>
       <c r="D3" s="3">
-        <v>481190.63450056087</v>
+        <v>2237559.59010129</v>
       </c>
       <c r="E3" s="3">
-        <v>5659.2905294400007</v>
+        <v>28962.7912646</v>
       </c>
       <c r="F3" s="4">
-        <v>2.7642536319032169E-4</v>
+        <v>0.18094518011478611</v>
       </c>
       <c r="G3" s="4">
-        <v>2.609783923120391E-3</v>
+        <v>2.339677504868966E-4</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2">
         <v>2022</v>
       </c>
       <c r="D4" s="3">
-        <v>463554.2380744408</v>
+        <v>2199098.9702055152</v>
       </c>
       <c r="E4" s="3">
-        <v>6405.1162323599992</v>
+        <v>27186.587841839999</v>
       </c>
       <c r="F4" s="4">
-        <v>1.36542870460566E-3</v>
+        <v>1.428164445640567E-2</v>
       </c>
       <c r="G4" s="4">
-        <v>1.06191448730258E-3</v>
+        <v>1.063284111568874E-3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D5" s="3">
-        <v>463215.01884109463</v>
+        <v>2136662.9096641121</v>
       </c>
       <c r="E5" s="3">
-        <v>6600.4823040000001</v>
+        <v>34419.6404244</v>
       </c>
       <c r="F5" s="4">
-        <v>1.0184783005820781E-3</v>
+        <v>1.2450489874850871E-3</v>
       </c>
       <c r="G5" s="4">
-        <v>1.1952508372333631E-3</v>
+        <v>2.6914455891389468E-4</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D6" s="3">
-        <v>624490.81179662514</v>
+        <v>2110825.0242093089</v>
       </c>
       <c r="E6" s="3">
-        <v>23490.718752000001</v>
+        <v>36820.330575920001</v>
       </c>
       <c r="F6" s="4">
-        <v>1.927088927244758E-3</v>
+        <v>1.1388913987487259E-2</v>
       </c>
       <c r="G6" s="4">
-        <v>1.8760825696850091E-3</v>
+        <v>1.346627653376551E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C7" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D7" s="3">
-        <v>615005.46689121344</v>
+        <v>2060147.693651289</v>
       </c>
       <c r="E7" s="3">
-        <v>18304.5266156</v>
+        <v>24111.565200000001</v>
       </c>
       <c r="F7" s="4">
-        <v>2.0544865338363899E-3</v>
+        <v>1.6816288641435851E-2</v>
       </c>
       <c r="G7" s="4">
-        <v>2.397692315221963E-3</v>
+        <v>4.7603910840263489E-4</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="D8" s="3">
-        <v>557880.96074185451</v>
+        <v>1963532.5336935241</v>
       </c>
       <c r="E8" s="3">
-        <v>17673.58753398</v>
+        <v>38266.632667600003</v>
       </c>
       <c r="F8" s="4">
-        <v>1.2639185721094849E-3</v>
+        <v>0.1254843771395045</v>
       </c>
       <c r="G8" s="4">
-        <v>7.224852054202324E-4</v>
+        <v>3.2594779133939081E-4</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="C9" s="2">
         <v>2022</v>
       </c>
       <c r="D9" s="3">
-        <v>528936.59684355662</v>
+        <v>1501058.080583167</v>
       </c>
       <c r="E9" s="3">
-        <v>14840.029964359999</v>
+        <v>10016.90090194</v>
       </c>
       <c r="F9" s="4">
-        <v>3.348617336982791E-3</v>
+        <v>4.8543989239808157E-3</v>
       </c>
       <c r="G9" s="4">
-        <v>9.7700369843055682E-4</v>
+        <v>2.722411311338672E-3</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D10" s="3">
-        <v>480752.63075950177</v>
+        <v>1438073.2884498299</v>
       </c>
       <c r="E10" s="3">
-        <v>13713.99982974</v>
+        <v>33002.728752000003</v>
       </c>
       <c r="F10" s="4">
-        <v>1.8909555433829729E-4</v>
+        <v>1.2530342781881009E-2</v>
       </c>
       <c r="G10" s="4">
-        <v>1.421912259449817E-2</v>
+        <v>4.7058508757579111E-4</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D11" s="3">
-        <v>430680.74778667098</v>
+        <v>1291276.529800517</v>
       </c>
       <c r="E11" s="3">
-        <v>9650.7308639999992</v>
+        <v>12420.628572240001</v>
       </c>
       <c r="F11" s="4">
-        <v>3.2382873836611008E-4</v>
+        <v>9.5505969516812179E-3</v>
       </c>
       <c r="G11" s="4">
-        <v>1.307147425181787E-3</v>
+        <v>7.1947529628030547E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D12" s="3">
-        <v>344818.33344279532</v>
+        <v>1235191.2922385989</v>
       </c>
       <c r="E12" s="3">
-        <v>7766.5175531200011</v>
+        <v>17766.839759999999</v>
       </c>
       <c r="F12" s="4">
-        <v>5.6879237956854514E-4</v>
+        <v>9.3958949512133153E-4</v>
       </c>
       <c r="G12" s="4">
-        <v>9.2862762115340628E-4</v>
+        <v>8.8262764857625984E-4</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C13" s="2">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D13" s="3">
-        <v>310794.74797233898</v>
+        <v>1202957.7138338401</v>
       </c>
       <c r="E13" s="3">
-        <v>8210.8821614400003</v>
+        <v>13409.25543712</v>
       </c>
       <c r="F13" s="4">
-        <v>1.515288413031857E-4</v>
+        <v>1.2431315547808089E-3</v>
       </c>
       <c r="G13" s="4">
-        <v>1.134724744407487E-2</v>
+        <v>1.4794270549193711E-3</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C14" s="2">
         <v>2024</v>
       </c>
       <c r="D14" s="3">
-        <v>615324.90182869229</v>
+        <v>1079590.799601601</v>
       </c>
       <c r="E14" s="3">
-        <v>12188.037840000001</v>
+        <v>29824.255583999999</v>
       </c>
       <c r="F14" s="4">
-        <v>3.5563801629943082E-3</v>
+        <v>1.7700063980245699E-2</v>
       </c>
       <c r="G14" s="4">
-        <v>2.3262126662383252E-3</v>
+        <v>1.8406361575525849E-2</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C15" s="2">
         <v>2023</v>
       </c>
       <c r="D15" s="3">
-        <v>463470.71898289572</v>
+        <v>917032.53729645221</v>
       </c>
       <c r="E15" s="3">
-        <v>9380.3853557600014</v>
+        <v>21948.7441788</v>
       </c>
       <c r="F15" s="4">
-        <v>2.4821681068467739E-3</v>
+        <v>5.1385668600091312E-2</v>
       </c>
       <c r="G15" s="4">
-        <v>1.7821392198706289E-3</v>
+        <v>1.045825844659099E-3</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C16" s="2">
         <v>2022</v>
       </c>
       <c r="D16" s="3">
-        <v>441905.15975913568</v>
+        <v>802566.08061441511</v>
       </c>
       <c r="E16" s="3">
-        <v>8680.9984719799995</v>
+        <v>12046.641059559999</v>
       </c>
       <c r="F16" s="4">
-        <v>5.3628300774693723E-2</v>
+        <v>1.264319260007594E-2</v>
       </c>
       <c r="G16" s="4">
-        <v>1.9809359137092151E-3</v>
+        <v>9.2646432850616075E-4</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C17" s="2">
         <v>2021</v>
       </c>
       <c r="D17" s="3">
-        <v>396416.47748978873</v>
+        <v>774599.50938466226</v>
       </c>
       <c r="E17" s="3">
-        <v>10615.43888874</v>
+        <v>31768.917493320001</v>
       </c>
       <c r="F17" s="4">
-        <v>5.7122249315871114E-3</v>
+        <v>4.5024994770462897E-3</v>
       </c>
       <c r="G17" s="4">
-        <v>1.223257961926933E-3</v>
+        <v>6.1504127372638605E-4</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18" s="2">
         <v>2024</v>
       </c>
       <c r="D18" s="3">
-        <v>333902.21266145178</v>
+        <v>702640.28510284843</v>
       </c>
       <c r="E18" s="3">
-        <v>6590.0541599999997</v>
+        <v>24692.815392</v>
       </c>
       <c r="F18" s="4">
-        <v>3.968817154607421E-3</v>
+        <v>1.2473785395074479E-2</v>
       </c>
       <c r="G18" s="4">
-        <v>1.4273582237145071E-3</v>
+        <v>1.210844187888221E-3</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C19" s="2">
         <v>2023</v>
       </c>
       <c r="D19" s="3">
-        <v>289865.32010952412</v>
+        <v>648523.59030139784</v>
       </c>
       <c r="E19" s="3">
-        <v>5130.8202951200001</v>
+        <v>20365.73930736</v>
       </c>
       <c r="F19" s="4">
-        <v>7.1409024001186736E-3</v>
+        <v>2.3285205202868371E-2</v>
       </c>
       <c r="G19" s="4">
-        <v>1.6292149323472839E-3</v>
+        <v>1.5783067550306741E-3</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C20" s="2">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="D20" s="3">
-        <v>259818.50988372459</v>
+        <v>624490.81179662514</v>
       </c>
       <c r="E20" s="3">
-        <v>45922.658233419999</v>
+        <v>23490.718752000001</v>
       </c>
       <c r="F20" s="4">
-        <v>4.0433840100499702E-5</v>
+        <v>1.927088927244758E-3</v>
       </c>
       <c r="G20" s="4">
-        <v>1.5232724169502069E-4</v>
+        <v>1.8760825696850091E-3</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C21" s="2">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D21" s="3">
-        <v>234189.89306239539</v>
+        <v>615324.90182869229</v>
       </c>
       <c r="E21" s="3">
-        <v>4733.3383234200001</v>
+        <v>12188.037840000001</v>
       </c>
       <c r="F21" s="4">
-        <v>6.6356632156617178E-4</v>
+        <v>3.5563801629943082E-3</v>
       </c>
       <c r="G21" s="4">
-        <v>3.1476572520248271E-3</v>
+        <v>2.3262126662383252E-3</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C22" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D22" s="3">
-        <v>702640.28510284843</v>
+        <v>615005.46689121344</v>
       </c>
       <c r="E22" s="3">
-        <v>24692.815392</v>
+        <v>18304.5266156</v>
       </c>
       <c r="F22" s="4">
-        <v>1.2473785395074479E-2</v>
+        <v>2.0544865338363899E-3</v>
       </c>
       <c r="G22" s="4">
-        <v>1.210844187888221E-3</v>
+        <v>2.397692315221963E-3</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C23" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D23" s="3">
-        <v>648523.59030139784</v>
+        <v>589836.07301855378</v>
       </c>
       <c r="E23" s="3">
-        <v>20365.73930736</v>
+        <v>3459.2387039999999</v>
       </c>
       <c r="F23" s="4">
-        <v>2.3285205202868371E-2</v>
+        <v>2.6129124854981389E-3</v>
       </c>
       <c r="G23" s="4">
-        <v>1.5783067550306741E-3</v>
+        <v>2.2962786554205951E-3</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C24" s="2">
         <v>2022</v>
       </c>
       <c r="D24" s="3">
-        <v>525586.90611574077</v>
+        <v>585427.26654459862</v>
       </c>
       <c r="E24" s="3">
-        <v>57596.7124071</v>
+        <v>4854.6591208600003</v>
       </c>
       <c r="F24" s="4">
-        <v>6.9328647193893768E-4</v>
+        <v>3.7612999688359748E-4</v>
       </c>
       <c r="G24" s="4">
-        <v>1.2640594598421069E-2</v>
+        <v>2.0756040556386131E-3</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C25" s="2">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="D25" s="3">
-        <v>489831.22166003252</v>
+        <v>575669.32501484314</v>
       </c>
       <c r="E25" s="3">
-        <v>28233.8392518</v>
+        <v>4774.9529707199999</v>
       </c>
       <c r="F25" s="4">
-        <v>1.7629362658082969E-3</v>
+        <v>2.8738600116371028E-4</v>
       </c>
       <c r="G25" s="4">
-        <v>1.091290811894655E-3</v>
+        <v>1.316480132589062E-3</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C26" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D26" s="3">
-        <v>1079590.799601601</v>
+        <v>557880.96074185451</v>
       </c>
       <c r="E26" s="3">
-        <v>29824.255583999999</v>
+        <v>17673.58753398</v>
       </c>
       <c r="F26" s="4">
-        <v>1.7700063980245699E-2</v>
+        <v>1.2639185721094849E-3</v>
       </c>
       <c r="G26" s="4">
-        <v>1.8406361575525849E-2</v>
+        <v>7.224852054202324E-4</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C27" s="2">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D27" s="3">
-        <v>917032.53729645221</v>
+        <v>532258.74860418728</v>
       </c>
       <c r="E27" s="3">
-        <v>21948.7441788</v>
+        <v>5998.8555937799993</v>
       </c>
       <c r="F27" s="4">
-        <v>5.1385668600091312E-2</v>
+        <v>3.3561812091085249E-3</v>
       </c>
       <c r="G27" s="4">
-        <v>1.045825844659099E-3</v>
+        <v>1.7434020366891251E-3</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C28" s="2">
         <v>2022</v>
       </c>
       <c r="D28" s="3">
-        <v>802566.08061441511</v>
+        <v>528936.59684355662</v>
       </c>
       <c r="E28" s="3">
-        <v>12046.641059559999</v>
+        <v>14840.029964359999</v>
       </c>
       <c r="F28" s="4">
-        <v>1.264319260007594E-2</v>
+        <v>3.348617336982791E-3</v>
       </c>
       <c r="G28" s="4">
-        <v>9.2646432850616075E-4</v>
+        <v>9.7700369843055682E-4</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C29" s="2">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D29" s="3">
-        <v>774599.50938466226</v>
+        <v>525586.90611574077</v>
       </c>
       <c r="E29" s="3">
-        <v>31768.917493320001</v>
+        <v>57596.7124071</v>
       </c>
       <c r="F29" s="4">
-        <v>4.5024994770462897E-3</v>
+        <v>6.9328647193893768E-4</v>
       </c>
       <c r="G29" s="4">
-        <v>6.1504127372638605E-4</v>
+        <v>1.2640594598421069E-2</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C30" s="2">
         <v>2021</v>
       </c>
       <c r="D30" s="3">
-        <v>2688475.9724428668</v>
+        <v>496312.33844584553</v>
       </c>
       <c r="E30" s="3">
-        <v>22918.622383440001</v>
+        <v>6058.6276942799996</v>
       </c>
       <c r="F30" s="4">
-        <v>1.411209606183382E-2</v>
+        <v>1.149126975828702E-3</v>
       </c>
       <c r="G30" s="4">
-        <v>6.7540592802753808E-4</v>
+        <v>4.3326889923906344E-3</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C31" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D31" s="3">
-        <v>2199098.9702055152</v>
+        <v>489831.22166003252</v>
       </c>
       <c r="E31" s="3">
-        <v>27186.587841839999</v>
+        <v>28233.8392518</v>
       </c>
       <c r="F31" s="4">
-        <v>1.428164445640567E-2</v>
+        <v>1.7629362658082969E-3</v>
       </c>
       <c r="G31" s="4">
-        <v>1.063284111568874E-3</v>
+        <v>1.091290811894655E-3</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="2">
+      <c r="A32" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="5">
         <v>2023</v>
       </c>
       <c r="D32" s="3">
-        <v>2110825.0242093089</v>
+        <v>481190.63450056087</v>
       </c>
       <c r="E32" s="3">
-        <v>36820.330575920001</v>
+        <v>5659.2905294400007</v>
       </c>
       <c r="F32" s="4">
-        <v>1.1388913987487259E-2</v>
+        <v>2.7642536319032169E-4</v>
       </c>
       <c r="G32" s="4">
-        <v>1.346627653376551E-3</v>
+        <v>2.609783923120391E-3</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C33" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D33" s="3">
-        <v>2060147.693651289</v>
+        <v>480752.63075950177</v>
       </c>
       <c r="E33" s="3">
-        <v>24111.565200000001</v>
+        <v>13713.99982974</v>
       </c>
       <c r="F33" s="4">
-        <v>1.6816288641435851E-2</v>
+        <v>1.8909555433829729E-4</v>
       </c>
       <c r="G33" s="4">
-        <v>4.7603910840263489E-4</v>
+        <v>1.421912259449817E-2</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C34" s="2">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D34" s="3">
-        <v>589836.07301855378</v>
+        <v>463554.2380744408</v>
       </c>
       <c r="E34" s="3">
-        <v>3459.2387039999999</v>
+        <v>6405.1162323599992</v>
       </c>
       <c r="F34" s="4">
-        <v>2.6129124854981389E-3</v>
+        <v>1.36542870460566E-3</v>
       </c>
       <c r="G34" s="4">
-        <v>2.2962786554205951E-3</v>
+        <v>1.06191448730258E-3</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C35" s="2">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D35" s="3">
-        <v>585427.26654459862</v>
+        <v>463470.71898289572</v>
       </c>
       <c r="E35" s="3">
-        <v>4854.6591208600003</v>
+        <v>9380.3853557600014</v>
       </c>
       <c r="F35" s="4">
-        <v>3.7612999688359748E-4</v>
+        <v>2.4821681068467739E-3</v>
       </c>
       <c r="G35" s="4">
-        <v>2.0756040556386131E-3</v>
+        <v>1.7821392198706289E-3</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C36" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D36" s="3">
-        <v>575669.32501484314</v>
+        <v>463215.01884109463</v>
       </c>
       <c r="E36" s="3">
-        <v>4774.9529707199999</v>
+        <v>6600.4823040000001</v>
       </c>
       <c r="F36" s="4">
-        <v>2.8738600116371028E-4</v>
+        <v>1.0184783005820781E-3</v>
       </c>
       <c r="G36" s="4">
-        <v>1.316480132589062E-3</v>
+        <v>1.1952508372333631E-3</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C37" s="2">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D37" s="3">
-        <v>532258.74860418728</v>
+        <v>441905.15975913568</v>
       </c>
       <c r="E37" s="3">
-        <v>5998.8555937799993</v>
+        <v>8680.9984719799995</v>
       </c>
       <c r="F37" s="4">
-        <v>3.3561812091085249E-3</v>
+        <v>5.3628300774693723E-2</v>
       </c>
       <c r="G37" s="4">
-        <v>1.7434020366891251E-3</v>
+        <v>1.9809359137092151E-3</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C38" s="2">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="D38" s="3">
-        <v>327266.01547195681</v>
+        <v>430680.74778667098</v>
       </c>
       <c r="E38" s="3">
-        <v>2736.7203125999999</v>
+        <v>9650.7308639999992</v>
       </c>
       <c r="F38" s="4">
-        <v>6.5575458761258591E-4</v>
+        <v>3.2382873836611008E-4</v>
       </c>
       <c r="G38" s="4">
-        <v>9.6186040198574876E-4</v>
+        <v>1.307147425181787E-3</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C39" s="2">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D39" s="3">
-        <v>323997.44760210218</v>
+        <v>396416.47748978873</v>
       </c>
       <c r="E39" s="3">
-        <v>2594.2840083999999</v>
+        <v>10615.43888874</v>
       </c>
       <c r="F39" s="4">
-        <v>4.4144095106468531E-4</v>
+        <v>5.7122249315871114E-3</v>
       </c>
       <c r="G39" s="4">
-        <v>4.2813564143465432E-3</v>
+        <v>1.223257961926933E-3</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C40" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D40" s="3">
-        <v>321762.90970591619</v>
+        <v>391236.03926557873</v>
       </c>
       <c r="E40" s="3">
-        <v>2793.945984</v>
+        <v>9174.7777388399991</v>
       </c>
       <c r="F40" s="4">
-        <v>3.0877619142976242E-4</v>
+        <v>7.2720955318134649E-3</v>
       </c>
       <c r="G40" s="4">
-        <v>1.0062327675981299E-3</v>
+        <v>4.0538663342816288E-4</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C41" s="2">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="D41" s="3">
-        <v>297602.00445720641</v>
+        <v>344818.33344279532</v>
       </c>
       <c r="E41" s="3">
-        <v>3256.4356082999998</v>
+        <v>7766.5175531200011</v>
       </c>
       <c r="F41" s="4">
-        <v>3.8592436982227681E-4</v>
+        <v>5.6879237956854514E-4</v>
       </c>
       <c r="G41" s="4">
-        <v>2.369477916386043E-3</v>
+        <v>9.2862762115340628E-4</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="C42" s="2">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D42" s="3">
-        <v>391236.03926557873</v>
+        <v>333902.21266145178</v>
       </c>
       <c r="E42" s="3">
-        <v>9174.7777388399991</v>
+        <v>6590.0541599999997</v>
       </c>
       <c r="F42" s="4">
-        <v>7.2720955318134649E-3</v>
+        <v>3.968817154607421E-3</v>
       </c>
       <c r="G42" s="4">
-        <v>4.0538663342816288E-4</v>
+        <v>1.4273582237145071E-3</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C43" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D43" s="3">
-        <v>331000.25434189721</v>
+        <v>332033.64455055603</v>
       </c>
       <c r="E43" s="3">
-        <v>7502.6813292799998</v>
+        <v>1720.9347523199999</v>
       </c>
       <c r="F43" s="4">
-        <v>1.753601618218082E-3</v>
+        <v>5.4438237053266124E-4</v>
       </c>
       <c r="G43" s="4">
-        <v>3.3407912051630981E-4</v>
+        <v>1.095196036606934E-3</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -1569,341 +1569,341 @@
         <v>18</v>
       </c>
       <c r="C44" s="2">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D44" s="3">
-        <v>315114.80271184049</v>
+        <v>331000.25434189721</v>
       </c>
       <c r="E44" s="3">
-        <v>3780.5631839999992</v>
+        <v>7502.6813292799998</v>
       </c>
       <c r="F44" s="4">
-        <v>1.04121883656369E-2</v>
+        <v>1.753601618218082E-3</v>
       </c>
       <c r="G44" s="4">
-        <v>1.4970467955548929E-3</v>
+        <v>3.3407912051630981E-4</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C45" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D45" s="3">
-        <v>311812.99097068148</v>
+        <v>327266.01547195681</v>
       </c>
       <c r="E45" s="3">
-        <v>3403.6800820799999</v>
+        <v>2736.7203125999999</v>
       </c>
       <c r="F45" s="4">
-        <v>7.8396110552474759E-4</v>
+        <v>6.5575458761258591E-4</v>
       </c>
       <c r="G45" s="4">
-        <v>1.35821810761219E-3</v>
+        <v>9.6186040198574876E-4</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C46" s="2">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D46" s="3">
-        <v>1501058.080583167</v>
+        <v>323997.44760210218</v>
       </c>
       <c r="E46" s="3">
-        <v>10016.90090194</v>
+        <v>2594.2840083999999</v>
       </c>
       <c r="F46" s="4">
-        <v>4.8543989239808157E-3</v>
+        <v>4.4144095106468531E-4</v>
       </c>
       <c r="G46" s="4">
-        <v>2.722411311338672E-3</v>
+        <v>4.2813564143465432E-3</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C47" s="2">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D47" s="3">
-        <v>1291276.529800517</v>
+        <v>321762.90970591619</v>
       </c>
       <c r="E47" s="3">
-        <v>12420.628572240001</v>
+        <v>2793.945984</v>
       </c>
       <c r="F47" s="4">
-        <v>9.5505969516812179E-3</v>
+        <v>3.0877619142976242E-4</v>
       </c>
       <c r="G47" s="4">
-        <v>7.1947529628030547E-3</v>
+        <v>1.0062327675981299E-3</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C48" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D48" s="3">
-        <v>1235191.2922385989</v>
+        <v>320449.11322310509</v>
       </c>
       <c r="E48" s="3">
-        <v>17766.839759999999</v>
+        <v>3164.1185242800002</v>
       </c>
       <c r="F48" s="4">
-        <v>9.3958949512133153E-4</v>
+        <v>6.7699852441129374E-3</v>
       </c>
       <c r="G48" s="4">
-        <v>8.8262764857625984E-4</v>
+        <v>2.6803313639870169E-3</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C49" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D49" s="3">
-        <v>1202957.7138338401</v>
+        <v>315114.80271184049</v>
       </c>
       <c r="E49" s="3">
-        <v>13409.25543712</v>
+        <v>3780.5631839999992</v>
       </c>
       <c r="F49" s="4">
-        <v>1.2431315547808089E-3</v>
+        <v>1.04121883656369E-2</v>
       </c>
       <c r="G49" s="4">
-        <v>1.4794270549193711E-3</v>
+        <v>1.4970467955548929E-3</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C50" s="2">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D50" s="3">
-        <v>2237559.59010129</v>
+        <v>311812.99097068148</v>
       </c>
       <c r="E50" s="3">
-        <v>28962.7912646</v>
+        <v>3403.6800820799999</v>
       </c>
       <c r="F50" s="4">
-        <v>0.18094518011478611</v>
+        <v>7.8396110552474759E-4</v>
       </c>
       <c r="G50" s="4">
-        <v>2.339677504868966E-4</v>
+        <v>1.35821810761219E-3</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C51" s="2">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D51" s="3">
-        <v>2136662.9096641121</v>
+        <v>310794.74797233898</v>
       </c>
       <c r="E51" s="3">
-        <v>34419.6404244</v>
+        <v>8210.8821614400003</v>
       </c>
       <c r="F51" s="4">
-        <v>1.2450489874850871E-3</v>
+        <v>1.515288413031857E-4</v>
       </c>
       <c r="G51" s="4">
-        <v>2.6914455891389468E-4</v>
+        <v>1.134724744407487E-2</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C52" s="2">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D52" s="3">
-        <v>1963532.5336935241</v>
+        <v>297602.00445720641</v>
       </c>
       <c r="E52" s="3">
-        <v>38266.632667600003</v>
+        <v>3256.4356082999998</v>
       </c>
       <c r="F52" s="4">
-        <v>0.1254843771395045</v>
+        <v>3.8592436982227681E-4</v>
       </c>
       <c r="G52" s="4">
-        <v>3.2594779133939081E-4</v>
+        <v>2.369477916386043E-3</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C53" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D53" s="3">
-        <v>1438073.2884498299</v>
+        <v>289865.32010952412</v>
       </c>
       <c r="E53" s="3">
-        <v>33002.728752000003</v>
+        <v>5130.8202951200001</v>
       </c>
       <c r="F53" s="4">
-        <v>1.2530342781881009E-2</v>
+        <v>7.1409024001186736E-3</v>
       </c>
       <c r="G53" s="4">
-        <v>4.7058508757579111E-4</v>
+        <v>1.6292149323472839E-3</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C54" s="2">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="D54" s="3">
-        <v>97959.145876195587</v>
+        <v>269939.47590449912</v>
       </c>
       <c r="E54" s="3">
-        <v>683.65838265999992</v>
+        <v>2592.956784</v>
       </c>
       <c r="F54" s="4">
-        <v>5.6993377084615887E-5</v>
+        <v>1.8052595511364291E-3</v>
       </c>
       <c r="G54" s="4">
-        <v>2.003412193486057E-3</v>
+        <v>8.4950123873718997E-4</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C55" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D55" s="3">
-        <v>95591.120637130909</v>
+        <v>262055.5197426404</v>
       </c>
       <c r="E55" s="3">
-        <v>1766.41918304</v>
+        <v>1735.1564722600001</v>
       </c>
       <c r="F55" s="4">
-        <v>1.0827214844375309E-3</v>
+        <v>3.0591654094954831E-3</v>
       </c>
       <c r="G55" s="4">
-        <v>1.157616504413661E-3</v>
+        <v>7.4264450532327117E-4</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C56" s="2">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D56" s="3">
-        <v>82867.321381128873</v>
+        <v>259818.50988372459</v>
       </c>
       <c r="E56" s="3">
-        <v>2276.6300928000001</v>
+        <v>45922.658233419999</v>
       </c>
       <c r="F56" s="4">
-        <v>2.6907058899788261E-3</v>
+        <v>4.0433840100499702E-5</v>
       </c>
       <c r="G56" s="4">
-        <v>8.8722397476340717E-4</v>
+        <v>1.5232724169502069E-4</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C57" s="2">
         <v>2021</v>
       </c>
       <c r="D57" s="3">
-        <v>320449.11322310509</v>
+        <v>234189.89306239539</v>
       </c>
       <c r="E57" s="3">
-        <v>3164.1185242800002</v>
+        <v>4733.3383234200001</v>
       </c>
       <c r="F57" s="4">
-        <v>6.7699852441129374E-3</v>
+        <v>6.6356632156617178E-4</v>
       </c>
       <c r="G57" s="4">
-        <v>2.6803313639870169E-3</v>
+        <v>3.1476572520248271E-3</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C58" s="2">
         <v>2024</v>
       </c>
       <c r="D58" s="3">
-        <v>269939.47590449912</v>
+        <v>208604.95707132079</v>
       </c>
       <c r="E58" s="3">
-        <v>2592.956784</v>
+        <v>1402.2910079999999</v>
       </c>
       <c r="F58" s="4">
-        <v>1.8052595511364291E-3</v>
+        <v>2.940331198358508E-3</v>
       </c>
       <c r="G58" s="4">
-        <v>8.4950123873718997E-4</v>
+        <v>9.1745863922704425E-4</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -1914,88 +1914,88 @@
         <v>8</v>
       </c>
       <c r="C59" s="2">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="D59" s="3">
-        <v>332033.64455055603</v>
+        <v>201018.8383422663</v>
       </c>
       <c r="E59" s="3">
-        <v>1720.9347523199999</v>
+        <v>1914.6587492000001</v>
       </c>
       <c r="F59" s="4">
-        <v>5.4438237053266124E-4</v>
+        <v>2.4675821537253392E-3</v>
       </c>
       <c r="G59" s="4">
-        <v>1.095196036606934E-3</v>
+        <v>4.9806477545852595E-4</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C60" s="2">
         <v>2022</v>
       </c>
       <c r="D60" s="3">
-        <v>262055.5197426404</v>
+        <v>97959.145876195587</v>
       </c>
       <c r="E60" s="3">
-        <v>1735.1564722600001</v>
+        <v>683.65838265999992</v>
       </c>
       <c r="F60" s="4">
-        <v>3.0591654094954831E-3</v>
+        <v>5.6993377084615887E-5</v>
       </c>
       <c r="G60" s="4">
-        <v>7.4264450532327117E-4</v>
+        <v>2.003412193486057E-3</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C61" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D61" s="3">
-        <v>208604.95707132079</v>
+        <v>95591.120637130909</v>
       </c>
       <c r="E61" s="3">
-        <v>1402.2910079999999</v>
+        <v>1766.41918304</v>
       </c>
       <c r="F61" s="4">
-        <v>2.940331198358508E-3</v>
+        <v>1.0827214844375309E-3</v>
       </c>
       <c r="G61" s="4">
-        <v>9.1745863922704425E-4</v>
+        <v>1.157616504413661E-3</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C62" s="2">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D62" s="3">
-        <v>201018.8383422663</v>
+        <v>82867.321381128873</v>
       </c>
       <c r="E62" s="3">
-        <v>1914.6587492000001</v>
+        <v>2276.6300928000001</v>
       </c>
       <c r="F62" s="4">
-        <v>2.4675821537253392E-3</v>
+        <v>2.6907058899788261E-3</v>
       </c>
       <c r="G62" s="4">
-        <v>4.9806477545852595E-4</v>
+        <v>8.8722397476340717E-4</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
@@ -2016,19 +2016,19 @@
       </c>
       <c r="D66" s="3">
         <f>AVERAGE(D2:D31)</f>
-        <v>655349.05308665475</v>
+        <v>1124212.4339560324</v>
       </c>
       <c r="E66" s="3">
         <f t="shared" ref="E66:G66" si="0">AVERAGE(E2:E31)</f>
-        <v>17273.303883399334</v>
+        <v>21247.447441487337</v>
       </c>
       <c r="F66" s="4">
         <f t="shared" si="0"/>
-        <v>8.1223329477286606E-3</v>
+        <v>1.7925682509706109E-2</v>
       </c>
       <c r="G66" s="4">
         <f t="shared" si="0"/>
-        <v>3.1965856646829407E-3</v>
+        <v>2.4906293556901716E-3</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
@@ -2037,19 +2037,19 @@
       </c>
       <c r="D67" s="3">
         <f>AVERAGE(D33:D62)</f>
-        <v>727998.75488181249</v>
+        <v>313456.52033605945</v>
       </c>
       <c r="E67" s="3">
         <f t="shared" ref="E67:G67" si="1">AVERAGE(E33:E62)</f>
-        <v>9465.4867188440021</v>
+        <v>6530.0444956386673</v>
       </c>
       <c r="F67" s="4">
         <f t="shared" si="1"/>
-        <v>1.3455747789443185E-2</v>
+        <v>4.0228145149423019E-3</v>
       </c>
       <c r="G67" s="4">
         <f t="shared" si="1"/>
-        <v>1.4843925181374825E-3</v>
+        <v>2.1482436181387908E-3</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
@@ -2058,19 +2058,19 @@
       </c>
       <c r="D69" s="3">
         <f>D66/D67</f>
-        <v>0.90020628289817317</v>
+        <v>3.5865019899753703</v>
       </c>
       <c r="E69" s="3">
         <f t="shared" ref="E69:G69" si="2">E66/E67</f>
-        <v>1.8248722328257498</v>
+        <v>3.2537982636532159</v>
       </c>
       <c r="F69" s="3">
         <f t="shared" si="2"/>
-        <v>0.60363296598804428</v>
+        <v>4.4560052279624465</v>
       </c>
       <c r="G69" s="3">
         <f t="shared" si="2"/>
-        <v>2.1534638753729403</v>
+        <v>1.1593793807464068</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
@@ -4566,8 +4566,8 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A149:G152">
-    <sortCondition descending="1" ref="D149:D152"/>
+  <sortState ref="A2:G62">
+    <sortCondition descending="1" ref="D2:D62"/>
   </sortState>
   <conditionalFormatting sqref="D2:D62">
     <cfRule type="colorScale" priority="128">

</xml_diff>